<commit_message>
Update BOM, clean up file structure, add init blender files
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3b86588c229cb83e/Documents/StudPrint/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="335" documentId="8_{09445066-EF4F-403A-BDCC-1386DA6612F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB4E2BEF-7DA1-434D-897D-058596732EE8}"/>
+  <xr:revisionPtr revIDLastSave="431" documentId="8_{09445066-EF4F-403A-BDCC-1386DA6612F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF607C82-6F3F-4BBE-BEC8-A4BF9AE42FB5}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{D2C1B5BA-DD01-4541-A6F5-99736AABD0EE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{D2C1B5BA-DD01-4541-A6F5-99736AABD0EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Off the shelf parts" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="127">
   <si>
     <t>Item</t>
   </si>
@@ -406,9 +406,6 @@
     <t>https://www.bricklink.com/v2/catalog/catalogitem.page?P=44728</t>
   </si>
   <si>
-    <t>NEED TO CHECK HOW MANY INVERTED</t>
-  </si>
-  <si>
     <t>https://www.bricklink.com/v2/catalog/catalogitem.page?P=73763</t>
   </si>
   <si>
@@ -428,6 +425,39 @@
   </si>
   <si>
     <t># Have</t>
+  </si>
+  <si>
+    <t>7.5</t>
+  </si>
+  <si>
+    <t>1x2_2x2_bracket Inverted</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>LEGO</t>
+  </si>
+  <si>
+    <t>Total Cost (CAD):</t>
+  </si>
+  <si>
+    <t>Total Cost (USD):</t>
+  </si>
+  <si>
+    <t>CHECK OTHER SHEET</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005010502837975.html</t>
+  </si>
+  <si>
+    <t>Ender 3 Limit Switch x3</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005002538357279.html</t>
+  </si>
+  <si>
+    <t>ECAS04</t>
   </si>
 </sst>
 </file>
@@ -502,7 +532,7 @@
       <name val="SWGDT"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -527,6 +557,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -542,7 +584,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -605,6 +647,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="44" fontId="0" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -645,10 +703,6 @@
     </a>
   </bag>
 </FeaturePropertyBags>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -968,7 +1022,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{267200E0-556E-48DA-9036-6ADBC4D5DBF8}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
@@ -1069,170 +1123,227 @@
       <c r="E5" s="24" t="b">
         <v>0</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A7" s="3" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" s="18">
+        <v>1</v>
+      </c>
+      <c r="C6" s="19">
+        <v>3.4</v>
+      </c>
+      <c r="D6" s="20">
+        <f>C6*B6</f>
+        <v>3.4</v>
+      </c>
+      <c r="E6" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A8" s="4" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B9" s="4">
         <v>4</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C9" s="5">
         <v>7.94</v>
       </c>
-      <c r="D8" s="6">
-        <f t="shared" ref="D8" si="0">B8*C8</f>
+      <c r="D9" s="6">
+        <f t="shared" ref="D9" si="0">B9*C9</f>
         <v>31.76</v>
       </c>
-      <c r="E8" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" s="8" t="s">
+      <c r="E9" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A10" s="9" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A11" s="13" t="s">
+      <c r="B11" s="10"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+    </row>
+    <row r="12" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="10">
-        <v>1</v>
-      </c>
-      <c r="C11" s="14">
+      <c r="B12" s="10">
+        <v>1</v>
+      </c>
+      <c r="C12" s="14">
         <v>14.67</v>
       </c>
-      <c r="D11" s="12">
-        <f>B11*C11</f>
+      <c r="D12" s="12">
+        <f>B12*C12</f>
         <v>14.67</v>
       </c>
-      <c r="E11" s="15" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" s="16" t="s">
+      <c r="E12" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="16" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="10">
-        <v>1</v>
-      </c>
-      <c r="C12" s="11">
-        <v>6.19</v>
-      </c>
-      <c r="D12" s="12">
-        <f>C12*B12</f>
-        <v>6.19</v>
-      </c>
-      <c r="E12" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="10">
+        <v>1</v>
+      </c>
+      <c r="C13" s="11">
+        <v>6.19</v>
+      </c>
+      <c r="D13" s="12">
+        <f>C13*B13</f>
+        <v>6.19</v>
+      </c>
+      <c r="E13" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A14" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="10">
-        <v>1</v>
-      </c>
-      <c r="C13" s="11">
+      <c r="B14" s="10">
+        <v>1</v>
+      </c>
+      <c r="C14" s="11">
         <v>7.03</v>
       </c>
-      <c r="D13" s="12">
-        <f t="shared" ref="D13" si="1">B13*C13</f>
+      <c r="D14" s="12">
+        <f t="shared" ref="D14" si="1">B14*C14</f>
         <v>7.03</v>
       </c>
-      <c r="E13" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" s="10" t="s">
+      <c r="E14" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="16" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="C14"/>
-      <c r="D14"/>
-    </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+      <c r="A15" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="10">
+        <v>1</v>
+      </c>
+      <c r="C15" s="11">
+        <v>2.48</v>
+      </c>
+      <c r="D15" s="12">
+        <f t="shared" ref="D15" si="2">B15*C15</f>
+        <v>2.48</v>
+      </c>
+      <c r="E15" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" s="37"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="39">
+        <f>LEGO!G33</f>
+        <v>26.665159999999993</v>
+      </c>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="2">
-        <f>SUM(D3:D13)</f>
-        <v>133.24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
+      <c r="D19" s="2">
+        <f>SUM(D3:D17)</f>
+        <v>165.78515999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="2">
-        <f>SUMIFS(D3:D13,E3:E13,TRUE)</f>
+      <c r="D21" s="2">
+        <f>SUMIFS(D3:D14,E3:E14,TRUE)</f>
         <v>46.43</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="2">
-        <f>D15-D17</f>
-        <v>86.81</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+      <c r="D22" s="2">
+        <f>D19-D21</f>
+        <v>119.35515999999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="2">
-        <f>D18*0.13</f>
-        <v>11.285300000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
+      <c r="D23" s="2">
+        <f>D22*0.13</f>
+        <v>15.516170799999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="2">
-        <f>D18+D19</f>
-        <v>98.095300000000009</v>
+      <c r="D24" s="2">
+        <f>D22+D23</f>
+        <v>134.87133079999998</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{A3995EEE-1759-4C86-98D6-DFEAD37C43E2}"/>
     <hyperlink ref="F4" r:id="rId2" xr:uid="{0408EDD3-F925-499A-8118-AC3EBC8F40C7}"/>
-    <hyperlink ref="F8" r:id="rId3" xr:uid="{A6E28D7D-7E0B-4C6F-BE7F-37CFED412A76}"/>
-    <hyperlink ref="F11" r:id="rId4" xr:uid="{4221E09E-D09B-4A82-A8A1-EA7EF10AA021}"/>
-    <hyperlink ref="F12" r:id="rId5" xr:uid="{2CACAE13-46CF-4C5B-A3A9-221B36B535A6}"/>
+    <hyperlink ref="F9" r:id="rId3" xr:uid="{A6E28D7D-7E0B-4C6F-BE7F-37CFED412A76}"/>
+    <hyperlink ref="F12" r:id="rId4" xr:uid="{4221E09E-D09B-4A82-A8A1-EA7EF10AA021}"/>
+    <hyperlink ref="F13" r:id="rId5" xr:uid="{2CACAE13-46CF-4C5B-A3A9-221B36B535A6}"/>
+    <hyperlink ref="F6" r:id="rId6" xr:uid="{335925B0-8D6F-4E56-87A8-5D802CFE6217}"/>
+    <hyperlink ref="F5" r:id="rId7" xr:uid="{621C3E9E-5F37-466D-849C-0D5C20AF04C2}"/>
+    <hyperlink ref="F14" r:id="rId8" xr:uid="{E725EF25-A042-4F7B-9775-6FC8C8ECF4A1}"/>
+    <hyperlink ref="F15" r:id="rId9" xr:uid="{D13FB5E7-CA00-423F-8F96-5CBB019F645C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1240,17 +1351,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{820EAF09-BA89-4E2F-B4BE-5324A1FD6D7F}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.1328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.3984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="54" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="14.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A1" s="28" t="s">
         <v>85</v>
       </c>
@@ -1264,13 +1376,16 @@
         <v>86</v>
       </c>
       <c r="E1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
+        <v>114</v>
+      </c>
+      <c r="G1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A2" s="28" t="s">
         <v>82</v>
       </c>
@@ -1283,8 +1398,18 @@
       <c r="D2" s="29" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="E2">
+        <v>14</v>
+      </c>
+      <c r="F2">
+        <f>C2-E2</f>
+        <v>34</v>
+      </c>
+      <c r="G2" s="1">
+        <v>5.85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A3" s="28" t="s">
         <v>81</v>
       </c>
@@ -1297,8 +1422,16 @@
       <c r="D3" s="29" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F30" si="0">C3-E3</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A4" s="28" t="s">
         <v>79</v>
       </c>
@@ -1311,8 +1444,16 @@
       <c r="D4" s="29" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="32.25" x14ac:dyDescent="0.45">
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" ht="32.25" x14ac:dyDescent="0.45">
       <c r="A5" s="28" t="s">
         <v>77</v>
       </c>
@@ -1323,10 +1464,20 @@
         <v>6</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
+        <v>113</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="G5" s="1">
+        <v>11.34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A6" s="28" t="s">
         <v>75</v>
       </c>
@@ -1339,8 +1490,16 @@
       <c r="D6" s="29" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="E6">
+        <v>30</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A7" s="28" t="s">
         <v>73</v>
       </c>
@@ -1353,8 +1512,16 @@
       <c r="D7" s="29" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A8" s="28" t="s">
         <v>71</v>
       </c>
@@ -1362,301 +1529,517 @@
         <v>68</v>
       </c>
       <c r="C8" s="26">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8">
+        <v>15</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30.75" x14ac:dyDescent="0.45">
+      <c r="A9" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="26">
+        <v>2</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A10" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="26">
+        <v>11</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10">
+        <v>11</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A11" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="26">
+        <v>15</v>
+      </c>
+      <c r="E11">
+        <v>15</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A12" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="26">
+        <v>14</v>
+      </c>
+      <c r="E12">
+        <v>14</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A13" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="26">
+        <v>18</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="E13">
+        <v>18</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A14" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="26">
+        <v>12</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="E14">
+        <v>12</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A15" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="26">
+        <v>20</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E15">
+        <v>20</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A16" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="26">
+        <v>1</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A17" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="26">
+        <v>3</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A18" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="32">
+        <v>4</v>
+      </c>
+      <c r="D18" s="33" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18" s="34">
+        <v>0</v>
+      </c>
+      <c r="F18" s="34">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="G18" s="35"/>
+    </row>
+    <row r="19" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A19" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="26">
+        <v>37</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="E19">
+        <v>37</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A20" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="26">
+        <v>16</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>101</v>
+      </c>
+      <c r="E20">
+        <v>16</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="1:7" ht="32.25" x14ac:dyDescent="0.45">
+      <c r="A21" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="26">
+        <v>13</v>
+      </c>
+      <c r="D21" s="29" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A9" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B9" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="26">
-        <v>11</v>
-      </c>
-      <c r="D9" s="29" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A10" s="28" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="26">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A11" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11" s="26">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A12" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" s="26">
-        <v>18</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A13" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="26">
-        <v>12</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A14" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="26">
-        <v>20</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A15" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" s="26">
-        <v>1</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A16" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="C16" s="26">
-        <v>3</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A17" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="26">
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="G21" s="1">
+        <v>17.16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A22" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="26">
         <v>4</v>
       </c>
-      <c r="D17" s="29" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A18" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="26">
+      <c r="D22" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22">
+        <v>4</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A23" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="26">
+        <v>6</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="E23">
+        <v>6</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A24" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="26">
+        <v>10</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E24">
+        <v>10</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A25" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" s="26">
+        <v>1</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A26" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="29" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A19" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="26">
-        <v>16</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="32.25" x14ac:dyDescent="0.45">
-      <c r="A20" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="26">
-        <v>13</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A21" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="26">
-        <v>4</v>
-      </c>
-      <c r="D21" s="29" t="s">
+      <c r="B26" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="26">
+        <v>1</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A27" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" s="26">
+        <v>2</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G27" s="1">
+        <v>1.464</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A28" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="26">
+        <v>1</v>
+      </c>
+      <c r="D28" s="29" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A22" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="26">
-        <v>6</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A23" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="26">
-        <v>10</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A24" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" s="26">
-        <v>1</v>
-      </c>
-      <c r="D24" s="29" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A25" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="C25" s="26">
-        <v>1</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A26" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="C26" s="26">
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A29" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="26">
+        <v>1</v>
+      </c>
+      <c r="D29" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A30" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="26">
         <v>2</v>
       </c>
-      <c r="D26" s="29" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A27" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="26">
-        <v>1</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A28" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="26">
-        <v>1</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A29" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="C29" s="26">
+      <c r="D30" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="E30">
         <v>2</v>
       </c>
-      <c r="D29" s="29" t="s">
-        <v>107</v>
+      <c r="F30">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="F32" t="s">
+        <v>120</v>
+      </c>
+      <c r="G32" s="36">
+        <f>SUM(G2:G30)</f>
+        <v>36.033999999999992</v>
+      </c>
+    </row>
+    <row r="33" spans="6:7" x14ac:dyDescent="0.45">
+      <c r="F33" t="s">
+        <v>121</v>
+      </c>
+      <c r="G33" s="36">
+        <f>G32*0.74</f>
+        <v>26.665159999999993</v>
       </c>
     </row>
   </sheetData>
@@ -1666,27 +2049,28 @@
     <hyperlink ref="D4" r:id="rId3" xr:uid="{B4F75F3E-8F01-4641-8441-572CA0332314}"/>
     <hyperlink ref="D6" r:id="rId4" xr:uid="{0BDB716C-8818-4949-91A4-C5FE8EA493E2}"/>
     <hyperlink ref="D7" r:id="rId5" xr:uid="{D66FD714-182C-4D45-9AA6-C9638D4A9CA2}"/>
-    <hyperlink ref="D9" r:id="rId6" xr:uid="{F07DCE8C-2BF5-4FC5-92C9-9F52F4F9D273}"/>
-    <hyperlink ref="D12" r:id="rId7" xr:uid="{1D785331-9977-4C0C-85A8-591CCC942060}"/>
-    <hyperlink ref="D13" r:id="rId8" xr:uid="{C129F461-B731-42DB-A1CD-0C6D588BEE3D}"/>
-    <hyperlink ref="D14" r:id="rId9" xr:uid="{4F932D1F-419F-494A-99B8-1C9E32890F7C}"/>
-    <hyperlink ref="D16" r:id="rId10" xr:uid="{9FEB77A8-84C1-4E8F-8EB9-FFC0C04D4095}"/>
-    <hyperlink ref="D15" r:id="rId11" xr:uid="{55BCBA33-23D4-4BA4-BAB3-A9A597209A1B}"/>
-    <hyperlink ref="D17" r:id="rId12" xr:uid="{B597B477-DE4A-4207-BA2D-C045C1585AAF}"/>
-    <hyperlink ref="D18" r:id="rId13" xr:uid="{ABE0C94C-AF79-4DE1-A1EB-07B5A7138CE3}"/>
-    <hyperlink ref="D19" r:id="rId14" xr:uid="{E07814CA-D017-4AB4-B7D9-E94357D6237D}"/>
-    <hyperlink ref="D22" r:id="rId15" xr:uid="{C7FAD275-0690-4777-8F98-DDFBBE9C9F04}"/>
-    <hyperlink ref="D23" r:id="rId16" xr:uid="{82012491-E67C-43BD-B524-A7326201A971}"/>
-    <hyperlink ref="D24" r:id="rId17" xr:uid="{053E921B-3913-4CC1-8CEA-7C9E17D81AB5}"/>
-    <hyperlink ref="D25" r:id="rId18" xr:uid="{5FB6AAFF-38C1-45E9-B6BA-DEE3A8C4A442}"/>
-    <hyperlink ref="D26" r:id="rId19" xr:uid="{FF265E5C-7DFF-441C-A4F8-94D7A544F820}"/>
-    <hyperlink ref="D29" r:id="rId20" xr:uid="{9BB5DFF6-FE91-4F6F-BF44-B622A11B7FC0}"/>
+    <hyperlink ref="D10" r:id="rId6" xr:uid="{F07DCE8C-2BF5-4FC5-92C9-9F52F4F9D273}"/>
+    <hyperlink ref="D13" r:id="rId7" xr:uid="{1D785331-9977-4C0C-85A8-591CCC942060}"/>
+    <hyperlink ref="D14" r:id="rId8" xr:uid="{C129F461-B731-42DB-A1CD-0C6D588BEE3D}"/>
+    <hyperlink ref="D15" r:id="rId9" xr:uid="{4F932D1F-419F-494A-99B8-1C9E32890F7C}"/>
+    <hyperlink ref="D17" r:id="rId10" xr:uid="{9FEB77A8-84C1-4E8F-8EB9-FFC0C04D4095}"/>
+    <hyperlink ref="D16" r:id="rId11" xr:uid="{55BCBA33-23D4-4BA4-BAB3-A9A597209A1B}"/>
+    <hyperlink ref="D18" r:id="rId12" xr:uid="{B597B477-DE4A-4207-BA2D-C045C1585AAF}"/>
+    <hyperlink ref="D19" r:id="rId13" xr:uid="{ABE0C94C-AF79-4DE1-A1EB-07B5A7138CE3}"/>
+    <hyperlink ref="D20" r:id="rId14" xr:uid="{E07814CA-D017-4AB4-B7D9-E94357D6237D}"/>
+    <hyperlink ref="D23" r:id="rId15" xr:uid="{C7FAD275-0690-4777-8F98-DDFBBE9C9F04}"/>
+    <hyperlink ref="D24" r:id="rId16" xr:uid="{82012491-E67C-43BD-B524-A7326201A971}"/>
+    <hyperlink ref="D25" r:id="rId17" xr:uid="{053E921B-3913-4CC1-8CEA-7C9E17D81AB5}"/>
+    <hyperlink ref="D26" r:id="rId18" xr:uid="{5FB6AAFF-38C1-45E9-B6BA-DEE3A8C4A442}"/>
+    <hyperlink ref="D27" r:id="rId19" xr:uid="{FF265E5C-7DFF-441C-A4F8-94D7A544F820}"/>
+    <hyperlink ref="D30" r:id="rId20" xr:uid="{9BB5DFF6-FE91-4F6F-BF44-B622A11B7FC0}"/>
     <hyperlink ref="D8" r:id="rId21" xr:uid="{477D9045-8750-48D4-8C46-3D15F2369764}"/>
-    <hyperlink ref="D21" r:id="rId22" xr:uid="{D22393AC-7F78-4041-806E-6D2B6F6DF870}"/>
-    <hyperlink ref="D20" r:id="rId23" xr:uid="{357FD862-4A22-42B2-BE66-B0C292B073F8}"/>
-    <hyperlink ref="D27" r:id="rId24" xr:uid="{32619FEF-A988-4AFA-AD79-4C03898FCE29}"/>
-    <hyperlink ref="D28" r:id="rId25" xr:uid="{68D25DFF-5DA6-435E-9E4A-E341EDD0A87C}"/>
+    <hyperlink ref="D22" r:id="rId22" xr:uid="{D22393AC-7F78-4041-806E-6D2B6F6DF870}"/>
+    <hyperlink ref="D21" r:id="rId23" xr:uid="{357FD862-4A22-42B2-BE66-B0C292B073F8}"/>
+    <hyperlink ref="D28" r:id="rId24" xr:uid="{32619FEF-A988-4AFA-AD79-4C03898FCE29}"/>
+    <hyperlink ref="D29" r:id="rId25" xr:uid="{68D25DFF-5DA6-435E-9E4A-E341EDD0A87C}"/>
     <hyperlink ref="D5" r:id="rId26" xr:uid="{36D58906-9761-47B7-92FB-F31BC23FCE0D}"/>
+    <hyperlink ref="D9" r:id="rId27" xr:uid="{8CFEFB2D-6297-44D3-844A-53F1270D542C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalize BOM, add RMRRF build improvements, add fasteners to CAD
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3b86588c229cb83e/Documents/StudPrint/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="520" documentId="8_{09445066-EF4F-403A-BDCC-1386DA6612F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCB3C5A8-8A8B-451D-8557-2FF0C3A1A243}"/>
+  <xr:revisionPtr revIDLastSave="608" documentId="8_{09445066-EF4F-403A-BDCC-1386DA6612F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63F9C2B5-A414-403D-B9E6-EF2FC9FB84E2}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{D2C1B5BA-DD01-4541-A6F5-99736AABD0EE}"/>
   </bookViews>
@@ -66,9 +66,6 @@
     <t>https://www.aliexpress.com/item/1005007038367315.html</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/1005008224603338.html</t>
-  </si>
-  <si>
     <t>https://www.aliexpress.com/item/1005006111249881.html</t>
   </si>
   <si>
@@ -115,9 +112,6 @@
   </si>
   <si>
     <t>https://www.aliexpress.com/item/1005010502837975.html</t>
-  </si>
-  <si>
-    <t>Ender 3 Limit Switch x3</t>
   </si>
   <si>
     <t>https://www.aliexpress.com/item/1005002538357279.html</t>
@@ -290,12 +284,6 @@
     <t>Bricklink URL</t>
   </si>
   <si>
-    <t>Axle 2L Notched</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
     <t>https://www.bricklink.com/catalogItem.asp?P=2456</t>
   </si>
   <si>
@@ -365,37 +353,69 @@
     <t>https://www.bricklink.com/catalogItem.asp?P=3034</t>
   </si>
   <si>
-    <t>Wheel Rim</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>Wheel Tire</t>
-  </si>
-  <si>
-    <t>https://www.bricklink.com/catalogItem.asp?P=92402</t>
-  </si>
-  <si>
     <t>https://www.bricklink.com/catalogItem.asp?P=4488</t>
   </si>
   <si>
-    <t>Wheel Connector</t>
-  </si>
-  <si>
-    <t>https://www.bricklink.com/catalogItem.asp?P=32062</t>
-  </si>
-  <si>
-    <t>Technic Worm Gear 6L</t>
-  </si>
-  <si>
     <t>https://www.bricklink.com/catalogItem.asp?P=48336</t>
   </si>
   <si>
     <t>Rough Estimate. Check other sheet for exact parts</t>
   </si>
   <si>
-    <t>Price in USD</t>
+    <t>wheel_connector</t>
+  </si>
+  <si>
+    <t>lego_wheel</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Technic Worm Gear </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="SWGDT"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>6L</t>
+    </r>
+  </si>
+  <si>
+    <t>Total LEGOs:</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005006023988927.html</t>
+  </si>
+  <si>
+    <t>Sherpa Mini Extruder Parts</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Ender 3 Limit Switch</t>
+  </si>
+  <si>
+    <t>Get the pack of 3</t>
+  </si>
+  <si>
+    <t>Only the drive gears and thumbscrew assembly is needed</t>
+  </si>
+  <si>
+    <t>Price in USD before tax and shipping</t>
+  </si>
+  <si>
+    <t>https://www.raspberrypi.com/products/raspberry-pi-zero-2-w/</t>
   </si>
 </sst>
 </file>
@@ -406,7 +426,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$$-1009]* #,##0.00_-;\-[$$-1009]* #,##0.00_-;_-[$$-1009]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -455,11 +475,6 @@
       <color theme="1"/>
       <name val="Century Gothic"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Century Gothic"/>
     </font>
     <font>
       <sz val="12"/>
@@ -557,12 +572,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -909,18 +920,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{267200E0-556E-48DA-9036-6ADBC4D5DBF8}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.06640625" customWidth="1"/>
     <col min="3" max="3" width="9.06640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.9296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.06640625" hidden="1"/>
+    <col min="5" max="5" width="48.9296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="48.9296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.06640625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -936,8 +949,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="15" t="s">
         <v>5</v>
       </c>
@@ -945,8 +961,9 @@
       <c r="C2" s="17"/>
       <c r="D2" s="18"/>
       <c r="E2" s="16"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F2" s="16"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="19" t="s">
         <v>7</v>
       </c>
@@ -963,8 +980,9 @@
       <c r="E3" s="20" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F3" s="20"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="19" t="s">
         <v>6</v>
       </c>
@@ -972,19 +990,20 @@
         <v>1</v>
       </c>
       <c r="C4" s="17">
-        <v>24.01</v>
+        <v>15</v>
       </c>
       <c r="D4" s="18">
         <f>B4*C4</f>
-        <v>24.01</v>
+        <v>15</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+        <v>112</v>
+      </c>
+      <c r="F4" s="20"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" s="16">
         <v>1</v>
@@ -997,12 +1016,13 @@
         <v>23.79</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+        <v>16</v>
+      </c>
+      <c r="F5" s="20"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="16" t="s">
-        <v>26</v>
+        <v>108</v>
       </c>
       <c r="B6" s="16">
         <v>1</v>
@@ -1015,21 +1035,28 @@
         <v>3.4</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+        <v>24</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="E7"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
       <c r="D8" s="6"/>
       <c r="E8" s="4"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="4">
         <v>4</v>
@@ -1042,21 +1069,26 @@
         <v>31.76</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+        <v>9</v>
+      </c>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="E10"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
       <c r="E11" s="9"/>
-    </row>
-    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A12" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="9">
         <v>1</v>
@@ -1069,12 +1101,13 @@
         <v>14.67</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+        <v>13</v>
+      </c>
+      <c r="F12" s="14"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13" s="9">
         <v>1</v>
@@ -1087,12 +1120,13 @@
         <v>7.94</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+        <v>9</v>
+      </c>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14" s="9">
         <v>1</v>
@@ -1105,12 +1139,13 @@
         <v>7.03</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+        <v>19</v>
+      </c>
+      <c r="F14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" s="9" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B15" s="9">
         <v>2</v>
@@ -1123,58 +1158,90 @@
         <v>4.96</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
+      </c>
+      <c r="F15" s="14"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="10">
+        <v>2.48</v>
+      </c>
+      <c r="D16" s="11">
+        <f t="shared" ref="D16" si="3">B16*C16</f>
+        <v>2.48</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="F16" s="30" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A17" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="28">
-        <v>30</v>
-      </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A18" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="26"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="28">
+        <v>60</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E19"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="2">
+        <f>SUM(D3:D18)</f>
+        <v>196.82</v>
+      </c>
+      <c r="E20" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="2">
-        <f>SUM(D3:D17)</f>
-        <v>173.35000000000002</v>
-      </c>
-      <c r="E19" t="s">
-        <v>112</v>
-      </c>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E22"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{A3995EEE-1759-4C86-98D6-DFEAD37C43E2}"/>
-    <hyperlink ref="E4" r:id="rId2" xr:uid="{0408EDD3-F925-499A-8118-AC3EBC8F40C7}"/>
-    <hyperlink ref="E9" r:id="rId3" xr:uid="{A6E28D7D-7E0B-4C6F-BE7F-37CFED412A76}"/>
-    <hyperlink ref="E12" r:id="rId4" xr:uid="{4221E09E-D09B-4A82-A8A1-EA7EF10AA021}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{335925B0-8D6F-4E56-87A8-5D802CFE6217}"/>
-    <hyperlink ref="E5" r:id="rId6" xr:uid="{621C3E9E-5F37-466D-849C-0D5C20AF04C2}"/>
-    <hyperlink ref="E14" r:id="rId7" xr:uid="{E725EF25-A042-4F7B-9775-6FC8C8ECF4A1}"/>
-    <hyperlink ref="E15" r:id="rId8" xr:uid="{D13FB5E7-CA00-423F-8F96-5CBB019F645C}"/>
-    <hyperlink ref="E13" r:id="rId9" xr:uid="{26CA49FA-4277-4FA5-A6B0-7A6BEB615727}"/>
+    <hyperlink ref="E9" r:id="rId1" xr:uid="{A6E28D7D-7E0B-4C6F-BE7F-37CFED412A76}"/>
+    <hyperlink ref="E12" r:id="rId2" xr:uid="{4221E09E-D09B-4A82-A8A1-EA7EF10AA021}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{621C3E9E-5F37-466D-849C-0D5C20AF04C2}"/>
+    <hyperlink ref="E14" r:id="rId4" xr:uid="{E725EF25-A042-4F7B-9775-6FC8C8ECF4A1}"/>
+    <hyperlink ref="E15" r:id="rId5" xr:uid="{D13FB5E7-CA00-423F-8F96-5CBB019F645C}"/>
+    <hyperlink ref="E13" r:id="rId6" xr:uid="{26CA49FA-4277-4FA5-A6B0-7A6BEB615727}"/>
+    <hyperlink ref="E16" r:id="rId7" xr:uid="{91E88391-35AE-4EAE-9C61-164B1DA540BE}"/>
+    <hyperlink ref="E6" r:id="rId8" xr:uid="{335925B0-8D6F-4E56-87A8-5D802CFE6217}"/>
+    <hyperlink ref="E3" r:id="rId9" xr:uid="{A3995EEE-1759-4C86-98D6-DFEAD37C43E2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId10"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{820EAF09-BA89-4E2F-B4BE-5324A1FD6D7F}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.9296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.9296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="54" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="14.46484375" bestFit="1" customWidth="1"/>
@@ -1182,171 +1249,171 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30.75" x14ac:dyDescent="0.45">
       <c r="A1" s="24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A2" s="24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C2" s="22">
         <v>48</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A3" s="24" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C3" s="22">
         <v>2</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A4" s="24" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C4" s="22">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A5" s="24" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C5" s="22">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A6" s="24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C6" s="22">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" ht="32.25" x14ac:dyDescent="0.45">
       <c r="A7" s="24" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C7" s="22">
         <v>6</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A8" s="24" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C8" s="22">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A9" s="24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C9" s="22">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A10" s="24" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C10" s="22">
         <v>14</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A11" s="24" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C11" s="22">
         <v>15</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A12" s="24" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B12" s="23" t="s">
         <v>102</v>
@@ -1355,275 +1422,301 @@
         <v>15</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A13" s="24" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>104</v>
+        <v>48</v>
       </c>
       <c r="C13" s="22">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A14" s="24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C14" s="22">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A15" s="24" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>54</v>
       </c>
       <c r="C15" s="22">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A16" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="29">
-        <v>40</v>
+      <c r="C16" s="22">
+        <v>3</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A17" s="24" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C17" s="22">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A18" s="24" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>65</v>
       </c>
       <c r="C18" s="22">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A19" s="24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B19" s="23" t="s">
         <v>67</v>
       </c>
       <c r="C19" s="22">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="32.25" x14ac:dyDescent="0.45">
       <c r="A20" s="24" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="C20" s="22">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" ht="30.75" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A21" s="24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="C21" s="22">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A22" s="24" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C22" s="22">
         <v>2</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A23" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="B23" s="30" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" s="29">
-        <v>2</v>
+        <v>61</v>
+      </c>
+      <c r="B23" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="22">
+        <v>1</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A24" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="B24" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="C24" s="29">
-        <v>1</v>
+        <v>62</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="22">
+        <v>5</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A25" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="B25" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="29">
-        <v>5</v>
+        <v>64</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="22">
+        <v>1</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A26" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="C26" s="29">
+        <v>66</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="22">
         <v>1</v>
       </c>
       <c r="D26" s="25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A27" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="C27" s="29">
-        <v>1</v>
-      </c>
-      <c r="D27" s="25" t="s">
-        <v>110</v>
-      </c>
+      <c r="A27" s="24"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="25"/>
     </row>
     <row r="28" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A28" s="24" t="s">
-        <v>103</v>
-      </c>
+      <c r="A28" s="24"/>
       <c r="B28" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="C28" s="22">
-        <v>9</v>
-      </c>
-      <c r="D28" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+        <v>104</v>
+      </c>
+      <c r="C28">
+        <f>SUM(C2:C26)</f>
+        <v>363</v>
+      </c>
+      <c r="D28" s="25"/>
+    </row>
+    <row r="29" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A29" s="24"/>
       <c r="D29" s="25"/>
     </row>
+    <row r="30" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A30" s="24"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="22"/>
+    </row>
+    <row r="31" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A31" s="24"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="22"/>
+    </row>
+    <row r="32" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A32" s="24"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="22"/>
+    </row>
+    <row r="33" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A33" s="24"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="22"/>
+    </row>
+    <row r="34" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A34" s="24"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="22"/>
+    </row>
+    <row r="35" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A35" s="24"/>
+    </row>
+    <row r="36" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A36" s="24"/>
+    </row>
+    <row r="37" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A37" s="24"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="22"/>
+    </row>
+    <row r="38" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A38" s="24"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="22"/>
+    </row>
+    <row r="39" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A39" s="24"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="22"/>
+    </row>
+    <row r="40" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A40" s="24"/>
+    </row>
+    <row r="41" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A41" s="24"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="22"/>
+    </row>
+    <row r="42" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A42" s="24"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="22"/>
+    </row>
+    <row r="43" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A43" s="24"/>
+    </row>
+    <row r="44" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A44" s="24"/>
+    </row>
   </sheetData>
-  <phoneticPr fontId="9" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{A2AB28BE-B4D6-43BC-9247-DD98CAB20AAC}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{801A8574-5A33-4AAD-8CE8-E0C333FE05F0}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{CEAF640A-EA43-40CF-9BEF-5EDF4DFA1C2F}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{ED924CF9-D841-4A5F-B0A2-14F1A9913B35}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{BE102573-F808-4A61-AC6A-34CDC73CAEC4}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{E97AB245-EF81-4BF4-8938-5C5AA8342256}"/>
-    <hyperlink ref="D8" r:id="rId7" xr:uid="{E2EAED41-E2A1-443B-A010-DE590C6DE5EA}"/>
-    <hyperlink ref="D9" r:id="rId8" xr:uid="{ED1918F4-71DE-402E-A1AF-2268F163CB7E}"/>
-    <hyperlink ref="D10" r:id="rId9" xr:uid="{EE4ABDA9-C3F2-49B0-857A-BC35A0760A2C}"/>
-    <hyperlink ref="D11" r:id="rId10" xr:uid="{4BFCA452-10F5-41DA-BA91-D6555A5BA5FB}"/>
-    <hyperlink ref="D12" r:id="rId11" xr:uid="{D2BE64A9-C51F-4695-95A2-B07B29AE8681}"/>
-    <hyperlink ref="D14" r:id="rId12" xr:uid="{48DE1FF0-C40B-41CB-BFC2-69198CB4A0FF}"/>
-    <hyperlink ref="D15" r:id="rId13" xr:uid="{5D2AB8A3-3862-4191-8E1D-51D58DDAB30F}"/>
-    <hyperlink ref="D16" r:id="rId14" xr:uid="{FAF463F8-A999-46BF-B6E5-55CC0A86A25C}"/>
-    <hyperlink ref="D17" r:id="rId15" xr:uid="{C5BB1B9D-0591-4362-8138-3F4A01418141}"/>
-    <hyperlink ref="D18" r:id="rId16" xr:uid="{6EEAA25B-F434-41F1-BE1C-749900E766F6}"/>
-    <hyperlink ref="D20" r:id="rId17" xr:uid="{2EA8F96C-8B72-4A02-AF22-AC38063915D7}"/>
-    <hyperlink ref="D21" r:id="rId18" xr:uid="{951078D8-F7C1-4A02-9ACE-3E0CFE29A375}"/>
-    <hyperlink ref="D22" r:id="rId19" xr:uid="{830C9809-B4FD-420A-88A4-024BE70E1FDD}"/>
-    <hyperlink ref="D23" r:id="rId20" xr:uid="{5465B1F9-E811-4179-BF5D-2FF087543415}"/>
-    <hyperlink ref="D24" r:id="rId21" xr:uid="{C4A06766-C643-4DD1-9306-D2187043025F}"/>
-    <hyperlink ref="D25" r:id="rId22" xr:uid="{EE493582-3A3B-488E-B2BB-7ACA91B11028}"/>
-    <hyperlink ref="D26" r:id="rId23" xr:uid="{CAD38CAC-56CF-404D-8509-DF6944050BCD}"/>
-    <hyperlink ref="D27" r:id="rId24" xr:uid="{C06D38BC-527D-4D47-B49A-CB9245B6B995}"/>
-    <hyperlink ref="D19" r:id="rId25" xr:uid="{F41F0905-2075-478F-97B9-9E24758BBC5F}"/>
-    <hyperlink ref="D13" r:id="rId26" xr:uid="{A062309D-5443-448C-B094-BC54B870EEBA}"/>
-    <hyperlink ref="D28" r:id="rId27" xr:uid="{152646EF-31E8-400C-81B3-4C6F43427D46}"/>
-  </hyperlinks>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>